<commit_message>
feat: import relational rows with durable ownership and safe recovery
</commit_message>
<xml_diff>
--- a/test/fixtures/files/conflict.xlsx
+++ b/test/fixtures/files/conflict.xlsx
@@ -489,16 +489,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="n">
-        <v>101</v>
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
           <t>Bramble Finch</t>
         </is>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>2</v>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>0000000000002</t>
+        </is>
       </c>
       <c r="D5" s="0"/>
       <c r="E5" s="0" t="inlineStr">
@@ -513,16 +517,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="n">
-        <v>108</v>
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
           <t>Conflicting Person</t>
         </is>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>1</v>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>0000000000001</t>
+        </is>
       </c>
       <c r="D6" s="0"/>
       <c r="E6" s="0" t="inlineStr">

</xml_diff>